<commit_message>
OMIEporra: datos del 2026-10-27
</commit_message>
<xml_diff>
--- a/omieporra_2026-10.xlsx
+++ b/omieporra_2026-10.xlsx
@@ -138,7 +138,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7435215" cy="4046220"/>
+    <ext cx="7463790" cy="4046220"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -448,11 +448,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -483,63 +483,6 @@
         <is>
           <t>Diferencia (€/MWh)</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Ejemplo Luis</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>82</v>
-      </c>
-      <c r="D2" t="n">
-        <v>158.68</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-76.68000000000001</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Ejemplo Ana</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="D3" t="n">
-        <v>158.68</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-83.18000000000001</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Ejemplo Marta</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>68.25</v>
-      </c>
-      <c r="D4" t="n">
-        <v>158.68</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-90.43000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -554,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1137,6 +1080,26 @@
         <v>158.68</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B29" t="n">
+        <v>96</v>
+      </c>
+      <c r="C29" t="n">
+        <v>197.46</v>
+      </c>
+      <c r="D29" t="n">
+        <v>57.08</v>
+      </c>
+      <c r="E29" t="n">
+        <v>319</v>
+      </c>
+      <c r="F29" t="n">
+        <v>160.06</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
OMIEporra: datos del 2026-10-28
</commit_message>
<xml_diff>
--- a/omieporra_2026-10.xlsx
+++ b/omieporra_2026-10.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1100,6 +1100,26 @@
         <v>160.06</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B30" t="n">
+        <v>96</v>
+      </c>
+      <c r="C30" t="n">
+        <v>231.01</v>
+      </c>
+      <c r="D30" t="n">
+        <v>115</v>
+      </c>
+      <c r="E30" t="n">
+        <v>322.78</v>
+      </c>
+      <c r="F30" t="n">
+        <v>162.51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
OMIEporra: datos del 2026-10-29
</commit_message>
<xml_diff>
--- a/omieporra_2026-10.xlsx
+++ b/omieporra_2026-10.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1120,6 +1120,26 @@
         <v>162.51</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B31" t="n">
+        <v>96</v>
+      </c>
+      <c r="C31" t="n">
+        <v>244.69</v>
+      </c>
+      <c r="D31" t="n">
+        <v>171.39</v>
+      </c>
+      <c r="E31" t="n">
+        <v>324.72</v>
+      </c>
+      <c r="F31" t="n">
+        <v>165.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
OMIEporra: datos del 2026-10-30
</commit_message>
<xml_diff>
--- a/omieporra_2026-10.xlsx
+++ b/omieporra_2026-10.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1140,6 +1140,26 @@
         <v>165.25</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B32" t="n">
+        <v>96</v>
+      </c>
+      <c r="C32" t="n">
+        <v>208.98</v>
+      </c>
+      <c r="D32" t="n">
+        <v>57.62</v>
+      </c>
+      <c r="E32" t="n">
+        <v>303.15</v>
+      </c>
+      <c r="F32" t="n">
+        <v>166.66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>